<commit_message>
The jupyter notebook workflow works. Adding to the geospatial workflow.
</commit_message>
<xml_diff>
--- a/src/LULUCF/scripts/postprocessing/LUC/conversion_LUC_scenario_results.xlsx
+++ b/src/LULUCF/scripts/postprocessing/LUC/conversion_LUC_scenario_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM27"/>
+  <dimension ref="A1:AM28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -970,9 +970,7 @@
       <c r="F4" t="b">
         <v>1</v>
       </c>
-      <c r="G4" t="b">
-        <v>1</v>
-      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
@@ -1026,52 +1024,52 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>forest_gmw_mangrove</t>
+          <t>forest_sdpt_planted_forest</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
@@ -1132,171 +1130,167 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
-        <v>2015</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>permanent_agriculture</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_gmw_mangrove</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="AM5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1315,161 +1309,159 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>crop_perm_ag_driver</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AL6" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="AM6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1477,7 +1469,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1488,30 +1480,32 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1521,7 +1515,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1531,7 +1525,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1541,106 +1535,106 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>grass_perm_ag_driver</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL7" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="AM7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1659,32 +1653,30 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="b">
-        <v>1</v>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1694,7 +1686,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -1704,7 +1696,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1714,27 +1706,27 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -1744,7 +1736,7 @@
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr">
@@ -1754,7 +1746,7 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1764,56 +1756,56 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="AM8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1821,41 +1813,43 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>2015</v>
+        <v>2020</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>shifting_cultivation</t>
+          <t>permanent_agriculture</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1865,7 +1859,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1875,7 +1869,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1885,27 +1879,27 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -1915,7 +1909,7 @@
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
@@ -1925,7 +1919,7 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1935,56 +1929,56 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="AM9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1996,7 +1990,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>logging</t>
+          <t>shifting_cultivation</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -2006,156 +2000,156 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_shift_cult_driver</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AL10" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="AM10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -2167,7 +2161,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>wildfire</t>
+          <t>logging</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -2177,156 +2171,156 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_logging_driver</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AL11" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="AM11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -2338,7 +2332,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>other_natural_disturbances</t>
+          <t>wildfire</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -2348,156 +2342,156 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_wildfire_driver</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="AM12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -2505,11 +2499,11 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>shifting_cultivation</t>
+          <t>other_natural_disturbances</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -2519,156 +2513,156 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>forest_nat_dist_driver</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="AM13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2680,7 +2674,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>logging</t>
+          <t>shifting_cultivation</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
@@ -2690,27 +2684,27 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -2720,7 +2714,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -2730,7 +2724,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -2740,27 +2734,27 @@
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
@@ -2770,7 +2764,7 @@
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
@@ -2780,7 +2774,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
@@ -2790,56 +2784,56 @@
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AI14" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL14" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="AM14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2851,7 +2845,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>wildfire</t>
+          <t>logging</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -2861,27 +2855,27 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2891,7 +2885,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2901,7 +2895,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2911,27 +2905,27 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
@@ -2941,7 +2935,7 @@
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
@@ -2951,7 +2945,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -2961,56 +2955,56 @@
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AI15" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL15" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="AM15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -3022,7 +3016,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>other_natural_disturbances</t>
+          <t>wildfire</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -3032,27 +3026,27 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -3062,7 +3056,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -3072,7 +3066,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -3082,27 +3076,27 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
@@ -3112,7 +3106,7 @@
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
@@ -3122,7 +3116,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -3132,64 +3126,70 @@
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AE16" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AI16" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL16" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="AM16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+      <c r="B17" t="n">
+        <v>2020</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>other_natural_disturbances</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
@@ -3197,321 +3197,317 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>forest</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>forest</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>forest</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>forest_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>forest_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>forest_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>other to forest</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>forest to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AI17" t="inlineStr">
         <is>
-          <t>other to forest</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>forest to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>other to forest</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL17" t="inlineStr">
         <is>
-          <t>other to forest to other to forest to other to forest</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="AM17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="n">
-        <v>2015</v>
-      </c>
+      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
-      <c r="D18" t="b">
-        <v>1</v>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
-          <t>cropland remaining cropland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>cropland remaining cropland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>cropland remaining cropland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>cropland remaining cropland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>cropland remaining cropland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>cropland remaining cropland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI18" t="inlineStr">
         <is>
-          <t>cropland remaining cropland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>cropland remaining cropland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>cropland remaining cropland</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="AM18" t="b">
@@ -3526,10 +3522,10 @@
         <v>2015</v>
       </c>
       <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="b">
+      <c r="D19" t="b">
         <v>1</v>
       </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
@@ -3585,52 +3581,52 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="AC19" t="inlineStr">
@@ -3692,13 +3688,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="C20" t="inlineStr"/>
-      <c r="D20" t="b">
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="b">
         <v>1</v>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
@@ -3754,52 +3750,52 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>crop_oil_palm</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="AC20" t="inlineStr">
@@ -3864,10 +3860,10 @@
         <v>2020</v>
       </c>
       <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="b">
+      <c r="D21" t="b">
         <v>1</v>
       </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
@@ -3923,52 +3919,52 @@
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>crop_sdpt_tree_crop</t>
+          <t>crop_oil_palm</t>
         </is>
       </c>
       <c r="AC21" t="inlineStr">
@@ -4029,165 +4025,169 @@
       <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="n">
+        <v>2020</v>
+      </c>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>crop_sdpt_tree_crop</t>
         </is>
       </c>
       <c r="AC22" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AD22" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AI22" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AK22" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AL22" t="inlineStr">
         <is>
-          <t>other to grassland to other to grassland to other to grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="AM22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -4203,37 +4203,37 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>forest</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -4253,37 +4253,37 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>forest_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
@@ -4293,7 +4293,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -4303,70 +4303,64 @@
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AD23" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>other to forest</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>forest to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AI23" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK23" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL23" t="inlineStr">
         <is>
-          <t>other to forest to other to grassland to other to grassland</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="AM23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>shifting_cultivation</t>
-        </is>
-      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
@@ -4374,27 +4368,27 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -4404,7 +4398,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -4414,7 +4408,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -4424,27 +4418,27 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
@@ -4454,7 +4448,7 @@
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
@@ -4464,7 +4458,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -4474,52 +4468,52 @@
       </c>
       <c r="AC24" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD24" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>other to forest</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
-          <t>forest to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI24" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest to grassland</t>
         </is>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK24" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL24" t="inlineStr">
         <is>
-          <t>other to forest to other to grassland to other to grassland</t>
+          <t>forest to grassland</t>
         </is>
       </c>
       <c r="AM24" t="b">
@@ -4530,8 +4524,14 @@
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
+      <c r="B25" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>shifting_cultivation</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
@@ -4539,27 +4539,27 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -4569,47 +4569,47 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>cropland</t>
+          <t>grassland</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
@@ -4619,72 +4619,72 @@
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>crop_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>crop_glad</t>
+          <t>grass_glad</t>
         </is>
       </c>
       <c r="AC25" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD25" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF25" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>other to forest</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>forest to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI25" t="inlineStr">
         <is>
-          <t>other to cropland</t>
+          <t>forest to grassland</t>
         </is>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>cropland to other</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AK25" t="inlineStr">
         <is>
-          <t>other to cropland</t>
+          <t>grassland remaining grassland</t>
         </is>
       </c>
       <c r="AL25" t="inlineStr">
         <is>
-          <t>other to forest to other to cropland to other to cropland</t>
+          <t>forest to grassland</t>
         </is>
       </c>
       <c r="AM25" t="b">
@@ -4695,14 +4695,8 @@
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>shifting_cultivation</t>
-        </is>
-      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
@@ -4710,27 +4704,27 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -4740,7 +4734,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -4750,7 +4744,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -4760,27 +4754,27 @@
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
@@ -4790,7 +4784,7 @@
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
@@ -4800,7 +4794,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_glad</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -4810,52 +4804,52 @@
       </c>
       <c r="AC26" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD26" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF26" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>other to forest</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>forest to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI26" t="inlineStr">
         <is>
-          <t>other to cropland</t>
+          <t>forest to cropland</t>
         </is>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
-          <t>cropland to other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AK26" t="inlineStr">
         <is>
-          <t>other to cropland</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AL26" t="inlineStr">
         <is>
-          <t>other to forest to other to cropland to other to cropland</t>
+          <t>forest to cropland</t>
         </is>
       </c>
       <c r="AM26" t="b">
@@ -4866,8 +4860,14 @@
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+      <c r="B27" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>shifting_cultivation</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
@@ -4875,27 +4875,27 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -4905,47 +4905,47 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>forest</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>grassland</t>
+          <t>cropland</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
@@ -4955,75 +4955,240 @@
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>forest_glad</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>crop_glad</t>
         </is>
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>bare_glad</t>
+          <t>crop_glad</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
-          <t>grass_glad</t>
+          <t>crop_glad</t>
         </is>
       </c>
       <c r="AC27" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AD27" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AE27" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AF27" t="inlineStr">
         <is>
-          <t>other remaining other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>other to forest</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>forest to other</t>
+          <t>forest remaining forest</t>
         </is>
       </c>
       <c r="AI27" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>forest to cropland</t>
         </is>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
-          <t>grassland to other</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AK27" t="inlineStr">
         <is>
-          <t>other to grassland</t>
+          <t>cropland remaining cropland</t>
         </is>
       </c>
       <c r="AL27" t="inlineStr">
         <is>
-          <t>other to forest to other to grassland to other to grassland</t>
+          <t>forest to cropland</t>
         </is>
       </c>
       <c r="AM27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>grassland</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>grassland</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>grassland</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>grassland</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>forest_glad</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>forest_glad</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>forest_glad</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>grass_glad</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>forest_glad</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>forest_glad</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>forest_glad</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr">
+        <is>
+          <t>grass_glad</t>
+        </is>
+      </c>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>grass_glad</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>grass_glad</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>forest remaining forest</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>forest remaining forest</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>forest to grassland</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>grassland to forest</t>
+        </is>
+      </c>
+      <c r="AG28" t="inlineStr">
+        <is>
+          <t>forest remaining forest</t>
+        </is>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>forest remaining forest</t>
+        </is>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>forest to grassland</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>grassland remaining grassland</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>grassland remaining grassland</t>
+        </is>
+      </c>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>forest to grassland to forest to grassland</t>
+        </is>
+      </c>
+      <c r="AM28" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>